<commit_message>
Refine assignment 3 assumption-aware tests
</commit_message>
<xml_diff>
--- a/workspace/assignment_3/Assignment_3_Statistical_Integrity_Tests.xlsx
+++ b/workspace/assignment_3/Assignment_3_Statistical_Integrity_Tests.xlsx
@@ -9,26 +9,32 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Box" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runs Test" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bollen Pool" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Negative Months" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Serial Tests" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autocorrelations" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lo Sharpe" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bias Ratio" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bias Bootstrap" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessment" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runs Exact Dist" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bollen Pool" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local Zero Bands" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bollen Bootstrap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Negative Months" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Serial Tests" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autocorrelations" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lo Sharpe" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bias Ratio" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bias Bootstrap" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessment" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data Box'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data Box'!$A$1:$I$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Runs Test'!$A$1:$M$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bollen Pool'!$A$1:$K$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Negative Months'!$A$1:$B$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Serial Tests'!$A$1:$I$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Autocorrelations'!$A$1:$D$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Lo Sharpe'!$A$1:$E$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Bias Ratio'!$A$1:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Bias Bootstrap'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Assessment'!$A$1:$D$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Runs Exact Dist'!$A$1:$D$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Bollen Pool'!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Local Zero Bands'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Bollen Bootstrap'!$A$1:$J$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Negative Months'!$A$1:$B$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Serial Tests'!$A$1:$I$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Autocorrelations'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Lo Sharpe'!$A$1:$E$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Bias Ratio'!$A$1:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Bias Bootstrap'!$A$1:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Assessment'!$A$1:$D$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,16 +459,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -488,15 +496,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>skewness</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>excess_kurtosis</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>positive</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>negative</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>sharpe</t>
         </is>
@@ -517,13 +535,19 @@
       <c r="D2" s="3" t="n">
         <v>4.010102220229272</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="3" t="n">
+        <v>2.649552522801263</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>8.518273050774795</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>108</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="H2" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="I2" s="3" t="n">
         <v>0.8716040257792279</v>
       </c>
     </row>
@@ -542,18 +566,24 @@
       <c r="D3" s="3" t="n">
         <v>4.543739913577447</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="3" t="n">
+        <v>-0.4507028811013243</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.5164587239200795</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="I3" s="3" t="n">
         <v>0.2921711009110291</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
+  <autoFilter ref="A1:I3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -564,11 +594,284 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>lags</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>monthly_sharpe</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>naive_annual_sharpe</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>lo_denominator</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>lo_adjusted_annual_sharpe</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>0.8716040257792279</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>3.019324913462393</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>2.930686502041501</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>1.763701842016465</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.8716040257792279</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>3.019324913462393</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>2.166594406950487</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>2.051261560606768</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Series</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>sigma</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>bias_ratio</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>expected_normal_br</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fund X</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>4.010102220229272</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>13.33333333333333</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>2.114798499335375</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 TR</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>4.543739913577447</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>repetitions</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>median</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>std</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>p5</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>observed_percentile</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>100000</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>20260625</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>15.2320989140031</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>13.16666666666667</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>8.601854590751968</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>28.66666666666667</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>51.939</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
   </cols>
@@ -603,7 +906,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>R=11, Rmax=11</t>
+          <t>R=11, exact lower-tail p=1.000</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -625,17 +928,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>p=4.64e-06</t>
+          <t>normal p=4.64e-06; local exact p=0.727</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Formal result is extreme</t>
+          <t>No local zero discontinuity</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Assumptions overstate significance</t>
+          <t>Normal count test is assumption-sensitive</t>
         </is>
       </c>
     </row>
@@ -657,7 +960,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Raw returns alone are misleading</t>
+          <t>p-values are approximate diagnostics</t>
         </is>
       </c>
     </row>
@@ -833,6 +1136,189 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>runs</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>probability</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>lower_tail_probability</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>upper_tail_probability</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>1.424861374524442e-08</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>1.424861374524442e-08</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>7.907980628610652e-07</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>8.050466766063096e-07</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.9999999857513863</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>6.098406682964611e-06</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>6.90345335957092e-06</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.9999991949533235</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.0001661815821107857</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.0001730850354703566</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0.9999930965466405</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.0004848233312956866</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.0006579083667660431</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.9998269149645297</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.008646016074773078</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.009303924441539121</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0.999342091633234</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0.01131254439689935</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.02061646883843847</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0.9906960755584608</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0.148477145209304</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0.1690936140477425</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0.9793835311615615</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0.0735315385798458</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.2426251526275883</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0.8309063859522575</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0.7573748473724117</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0.7573748473724117</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -986,7 +1472,248 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>band_percent</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>small_positive</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>small_negative</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>near_zero_total</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>positive_share</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>one_sided_p_too_many_positive</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>two_sided_exact_p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.36328125</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.7265625</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.0007448196411132812</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.001489639282226562</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>repetitions</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>block_length</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>observed_negative_months</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>mean_negative_months</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>median_negative_months</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>p5_negative_months</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>p95_negative_months</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>empirical_lower_tail_probability</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>empirical_upper_tail_probability</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>100000</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>5.00218</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.61498</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0.5602200000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1067,7 +1794,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1229,7 +1956,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1438,277 +2165,4 @@
   <autoFilter ref="A1:D13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="27" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>lags</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>monthly_sharpe</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>naive_annual_sharpe</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>lo_denominator</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>lo_adjusted_annual_sharpe</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>0.8716040257792279</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>3.019324913462393</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>2.930686502041501</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>1.763701842016465</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>0.8716040257792279</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>3.019324913462393</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>2.166594406950487</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>2.051261560606768</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E3"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Series</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>sigma</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>bias_ratio</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>expected_normal_br</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Fund X</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>4.010102220229272</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>13.33333333333333</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>2.114798499335375</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 500 TR</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>4.543739913577447</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>2.85</v>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F3"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>repetitions</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>seed</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>median</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>std</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>p5</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>p95</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>observed_percentile</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>100000</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>20260625</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>15.2320989140031</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>13.16666666666667</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>8.601854590751968</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>28.66666666666667</v>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>51.939</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:H2"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>